<commit_message>
feat(F-NAR-009): SAN/HYG/MOV/SOM et ramifiées COL-005–030
Ouvertures monde d’abord, chacune différente. Audio plus tard.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-REL.PAR.002-08.xlsx
+++ b/stories/arbres/ATOM-REL.PAR.002-08.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ferdinand attend la balançoire</t>
+          <t>Chouchou attend la balançoire</t>
         </is>
       </c>
     </row>
@@ -602,6 +602,11 @@
           <t>secondary_lessons</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>REL.PAR.001</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -830,6 +835,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Une coccinelle marche sur le banc. Les bottes de Chouchou font couic. Nina se balance. Chouchou attend. Puis c'est son tour.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand est au parc. Papa est près. Lila est sur la balançoire. La chaîne cliquette. Ferdinand a envie. Il s'approche. On attend. Ferdinand attend. Il pose les pieds au sol. Il compte. Un. Deux. Trois. Lila se balance encore. Ferdinand attend. Le bois de la barre est lisse. Lila descend. Puis mon tour. Puis mon tour. Il s'assoit. Il se balance. Ses mains tiennent la chaîne. Lila attend maintenant. Papa sourit.</t>
+          <t>Une coccinelle marche sur le banc. Le bois est encore un peu mouillé. La pluie a fini, tout à l'heure. Ça sent la terre douce. Derrière le parc, une petite maison. Chouchou habite ici, avec papa. Maman range les chaussettes, tout près. Les bottes de Chouchou font couic. Elles sont jaunes, un peu lourdes. Tu as vu la coccinelle, Chouchou ? Elle marche, papa. Oui. Elle a des points noirs. On pose tes bottes près du banc ? Oui, papa. Chouchou pose ses bottes. Ses chaussettes sont chaudes, tout douces. La coccinelle avance encore. Elle va tout doux, hein ? Tout doux. En ce moment, ils sont près de la balançoire. Le bois de la barre est lisse. Nina est sur la balançoire. La chaîne cliquette, tout doux. Nina se balance encore. Chouchou a envie de la balançoire. Papa, je veux me balancer. On attend. Nina finit. Puis c'est ton tour. Chouchou pose les pieds au sol. Il reste près de papa. Il compte tout bas. Un. Deux. Trois. Nina se balance encore un peu. Chouchou attend. Tu attends bien, Chouchou. Tes pieds sont au sol. Bravo. La coccinelle arrive au bord. Tu l'as vue, encore ? Oui, papa. Le bois de la barre brille. Chouchou attend encore. On reste près. Puis ce sera ton tour. Nina ralentit. La chaîne se tait un peu. Chouchou serre la main de papa. Encore un peu. Puis ton tour. Une feuille tombe près des bottes. Tu l'as vue, la feuille ? Oui. Elle tourne. On attend encore un tout petit peu. Chouchou souffle. Il reste près de papa. Tu attends. Bravo.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,12 +1329,67 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Ferdinand est au parc. Papa est près. Lila est sur la balançoire. La chaîne cliquette. Ferdinand a envie. Il s'approche.
+          <t>narrateur|Une coccinelle marche sur le banc.
+narrateur|Le bois est encore un peu mouillé.
+narrateur|La pluie a fini, tout à l'heure.
+narrateur|Ça sent la terre douce.
+narrateur|Derrière le parc, une petite maison.
+narrateur|Chouchou habite ici, avec papa.
+narrateur|Maman range les chaussettes, tout près.
+narrateur|Les bottes de Chouchou font couic.
+narrateur|Elles sont jaunes, un peu lourdes.
+papa|Tu as vu la coccinelle, Chouchou ?
+enfant-m|Elle marche, papa.
+papa|Oui.
+papa|Elle a des points noirs.
+papa|On pose tes bottes près du banc ?
+enfant-m|Oui, papa.
+narrateur|Chouchou pose ses bottes.
+narrateur|Ses chaussettes sont chaudes, tout douces.
+narrateur|La coccinelle avance encore.
+papa|Elle va tout doux, hein ?
+enfant-m|Tout doux.
+narrateur|En ce moment, ils sont près de la balançoire.
+narrateur|Le bois de la barre est lisse.
+narrateur|Nina est sur la balançoire.
+narrateur|La chaîne cliquette, tout doux.
+narrateur|Nina se balance encore.
+narrateur|Chouchou a envie de la balançoire.
+enfant-m|Papa, je veux me balancer.
 papa|On attend.
-narrateur|Ferdinand attend. Il pose les pieds au sol. Il compte. Un. Deux. Trois. Lila se balance encore. Ferdinand attend. Le bois de la barre est lisse. Lila descend.
-papa|Puis mon tour.
-enfant-m|Puis mon tour.
-narrateur|Il s'assoit. Il se balance. Ses mains tiennent la chaîne. Lila attend maintenant. Papa sourit.</t>
+papa|Nina finit.
+papa|Puis c'est ton tour.
+narrateur|Chouchou pose les pieds au sol.
+narrateur|Il reste près de papa.
+narrateur|Il compte tout bas.
+enfant-m|Un.
+enfant-m|Deux.
+enfant-m|Trois.
+narrateur|Nina se balance encore un peu.
+narrateur|Chouchou attend.
+papa|Tu attends bien, Chouchou.
+papa|Tes pieds sont au sol.
+papa|Bravo.
+narrateur|La coccinelle arrive au bord.
+papa|Tu l'as vue, encore ?
+enfant-m|Oui, papa.
+narrateur|Le bois de la barre brille.
+narrateur|Chouchou attend encore.
+papa|On reste près.
+papa|Puis ce sera ton tour.
+narrateur|Nina ralentit.
+narrateur|La chaîne se tait un peu.
+narrateur|Chouchou serre la main de papa.
+papa|Encore un peu.
+papa|Puis ton tour.
+narrateur|Une feuille tombe près des bottes.
+papa|Tu l'as vue, la feuille ?
+enfant-m|Oui.
+enfant-m|Elle tourne.
+papa|On attend encore un tout petit peu.
+narrateur|Chouchou souffle.
+narrateur|Il reste près de papa.
+papa|Tu attends. Bravo.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1349,7 +1421,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Lila est sur la balançoire. Que fait Ferdinand ?</t>
+          <t>Nina est sur la balançoire. Que fait Chouchou ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1505,7 +1577,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Lila est sur la balançoire. Que fait Ferdinand ?</t>
+          <t>narrateur|Nina est sur la balançoire.
+narrateur|Que fait Chouchou ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1533,7 +1606,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand a su attendre. Puis mon tour est venu. Il s'est balancé. Papa est là.</t>
+          <t>Nina descend. Maintenant. Puis c'est ton tour. Puis mon tour. Chouchou s'assoit. Il se balance. Ses mains tiennent la chaîne. La chaîne chante un peu. Bravo, Chouchou. Tu as attendu. C'est du bon travail. La chaîne est froide, papa. Oui. Elle se réchauffe. Nina attend maintenant, près du banc. Tu as su attendre. Chouchou va et vient, tout doux. Tu te balances tout doux. Le vent pousse un peu. Ça chatouille, papa. Oui. Le vent t'aide. Parce que tu as attendu, c'est ton tour. Nina reste près du banc. La coccinelle n'est plus là.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1677,7 +1750,30 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Ferdinand a su attendre. Puis mon tour est venu. Il s'est balancé. Papa est là.</t>
+          <t>narrateur|Nina descend.
+papa|Maintenant.
+papa|Puis c'est ton tour.
+enfant-m|Puis mon tour.
+narrateur|Chouchou s'assoit.
+narrateur|Il se balance.
+narrateur|Ses mains tiennent la chaîne.
+narrateur|La chaîne chante un peu.
+papa|Bravo, Chouchou.
+papa|Tu as attendu.
+papa|C'est du bon travail.
+enfant-m|La chaîne est froide, papa.
+papa|Oui.
+papa|Elle se réchauffe.
+narrateur|Nina attend maintenant, près du banc.
+papa|Tu as su attendre.
+narrateur|Chouchou va et vient, tout doux.
+papa|Tu te balances tout doux.
+narrateur|Le vent pousse un peu.
+enfant-m|Ça chatouille, papa.
+papa|Oui. Le vent t'aide.
+papa|Parce que tu as attendu, c'est ton tour.
+narrateur|Nina reste près du banc.
+narrateur|La coccinelle n'est plus là.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1705,7 +1801,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand range son manteau. Il prend la main de papa.</t>
+          <t>Chouchou descend. Tu veux laisser la balançoire à Nina ? Oui, papa. Bravo. On peut prêter. Nina reprend la balançoire. Chouchou prend la main de papa. On reprend tes bottes ? Oui. Les bottes sont un peu fraîches. Tu as bien attendu, Chouchou. Puis c'était mon tour. Oui. Puis ton tour. La coccinelle n'est plus sur le banc. On rentre ? Oui, papa. La balançoire se tait.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1845,7 +1941,24 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ferdinand range son manteau. Il prend la main de papa.</t>
+          <t>narrateur|Chouchou descend.
+papa|Tu veux laisser la balançoire à Nina ?
+enfant-m|Oui, papa.
+papa|Bravo.
+papa|On peut prêter.
+narrateur|Nina reprend la balançoire.
+narrateur|Chouchou prend la main de papa.
+papa|On reprend tes bottes ?
+enfant-m|Oui.
+narrateur|Les bottes sont un peu fraîches.
+papa|Tu as bien attendu, Chouchou.
+enfant-m|Puis c'était mon tour.
+papa|Oui.
+papa|Puis ton tour.
+narrateur|La coccinelle n'est plus sur le banc.
+papa|On rentre ?
+enfant-m|Oui, papa.
+narrateur|La balançoire se tait.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1873,7 +1986,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>J'ai attendu. Puis je me suis balancé. Bravo. Tu as fait du bon travail. Les bottes jaunes attendent près de la porte. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2013,7 +2126,12 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-m|J'ai attendu.
+enfant-m|Puis je me suis balancé.
+papa|Bravo.
+papa|Tu as fait du bon travail.
+narrateur|Les bottes jaunes attendent près de la porte.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2035,7 +2153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2073,6 +2191,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>